<commit_message>
Continuing my restructuring. Actually wrote a README to give myself a plan lol
</commit_message>
<xml_diff>
--- a/backend/API_Weather/excel_CSV_weather_stations.xlsx
+++ b/backend/API_Weather/excel_CSV_weather_stations.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\willh\water_dashboard\backend\API_Weather\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F1FB7B8-DF86-4C1F-B198-51EBCDAEC38C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C240AB5B-2B81-4DD9-AC5B-28AFD400C81C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C6EA2CE3-1894-40F2-9905-F0A661A0A308}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C6EA2CE3-1894-40F2-9905-F0A661A0A308}"/>
   </bookViews>
   <sheets>
     <sheet name="CSV_weather_stations" sheetId="1" r:id="rId1"/>
@@ -405,7 +405,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="35">
+  <fills count="36">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -594,6 +594,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -758,13 +764,15 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="22" fontId="0" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="22" fontId="0" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="22" fontId="0" fillId="35" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1192,8 +1200,8 @@
     <col min="1" max="1" width="9.28515625" customWidth="1"/>
     <col min="2" max="2" width="26.42578125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="20.85546875" customWidth="1"/>
-    <col min="4" max="4" width="18.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.28515625" hidden="1" customWidth="1"/>
+    <col min="5" max="5" width="15.5703125" hidden="1" customWidth="1"/>
     <col min="6" max="6" width="17.140625" customWidth="1"/>
     <col min="7" max="7" width="16.42578125" customWidth="1"/>
     <col min="8" max="8" width="18.28515625" bestFit="1" customWidth="1"/>
@@ -1257,10 +1265,10 @@
       <c r="A2">
         <v>27211</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="C2" s="2">
+      <c r="C2" s="6">
         <v>3031094</v>
       </c>
       <c r="D2" s="3">
@@ -1275,10 +1283,10 @@
       <c r="G2" s="3">
         <v>46243.520949074074</v>
       </c>
-      <c r="H2" s="3">
+      <c r="H2" s="7">
         <v>36281</v>
       </c>
-      <c r="I2" s="3">
+      <c r="I2" s="7">
         <v>46243</v>
       </c>
       <c r="J2" s="3">
@@ -3483,8 +3491,9 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>